<commit_message>
Fixed verification and validatio cases
</commit_message>
<xml_diff>
--- a/tests/Verification/core_case_ranges.xlsx
+++ b/tests/Verification/core_case_ranges.xlsx
@@ -499,12 +499,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>177.326 to 190.801</t>
+          <t>162.099 to 172.894</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>847.275 to 865.642</t>
+          <t>845.824 to 862.939</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>167.133 to 193.81</t>
+          <t>161.037 to 184.132</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -557,12 +557,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2352.42 to 5986.57</t>
+          <t>2352.42 to 4039.12</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0340668 to 0.0866951</t>
+          <t>0.0504919 to 0.0866951</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>160.022 to 218.565</t>
+          <t>160.022 to 170.187</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>834.803 to 913.57</t>
+          <t>834.803 to 851.565</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>183.323 to 194.087</t>
+          <t>172.173 to 185.625</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>861.075 to 883.245</t>
+          <t>848.116 to 869.979</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -691,22 +691,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>181.636 to 227.87</t>
+          <t>171.916 to 194.079</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>854.006 to 907.855</t>
+          <t>848.861 to 892.665</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3297.91 to 15477.7</t>
+          <t>3084.2 to 7024.57</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.0131766 to 0.0618402</t>
+          <t>0.0290329 to 0.0661251</t>
         </is>
       </c>
     </row>
@@ -735,16 +735,16 @@
         <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>177.138 to 197.23</t>
+          <t>170.269 to 188.291</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>848.522 to 903.326</t>
+          <t>836.939 to 884.609</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -783,16 +783,16 @@
         <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>191.116 to 200.307</t>
+          <t>171.79 to 185.314</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>884.236 to 909.284</t>
+          <t>847.505 to 869.284</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -835,22 +835,22 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>191.667 to 229.918</t>
+          <t>171.444 to 193.693</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>857.553 to 939.835</t>
+          <t>848.19 to 891.244</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3987.57 to 16103.9</t>
+          <t>3084.2 to 6984.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.0126642 to 0.0511447</t>
+          <t>0.0291982 to 0.0661251</t>
         </is>
       </c>
     </row>
@@ -879,16 +879,16 @@
         <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>188.803 to 213.489</t>
+          <t>169.858 to 187.906</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>874.077 to 969.758</t>
+          <t>836.319 to 883.358</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0.0373865 to 0.0373866</t>
+          <t>0.0373865 to 0.0373865</t>
         </is>
       </c>
     </row>
@@ -931,12 +931,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>173.759 to 186.634</t>
+          <t>158.987 to 169.059</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>847.27 to 865.603</t>
+          <t>845.811 to 862.82</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>164.057 to 189.403</t>
+          <t>158.147 to 180.087</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2342.11 to 5968.78</t>
+          <t>2342.11 to 3978.5</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>0.0341683 to 0.0870766</t>
+          <t>0.0512613 to 0.0870766</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>157.034 to 213.307</t>
+          <t>157.035 to 166.393</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>834.781 to 913.98</t>
+          <t>834.781 to 851.026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>179.248 to 189.518</t>
+          <t>168.429 to 181.031</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>861.015 to 882.983</t>
+          <t>848.035 to 869.687</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>177.558 to 221.585</t>
+          <t>168.193 to 189.438</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>854.029 to 908.01</t>
+          <t>848.914 to 892.744</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3277.34 to 15344</t>
+          <t>3067.06 to 6859.36</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>0.0132914 to 0.0622282</t>
+          <t>0.0297321 to 0.0664946</t>
         </is>
       </c>
     </row>
@@ -1167,16 +1167,16 @@
         <v>36</v>
       </c>
       <c r="F16" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>173.06 to 191.941</t>
+          <t>166.623 to 183.317</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>848.328 to 901.388</t>
+          <t>836.843 to 882.777</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>186.573 to 194.913</t>
+          <t>168.062 to 180.73</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>884.082 to 908.769</t>
+          <t>847.412 to 868.978</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1267,22 +1267,22 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>187.04 to 223.529</t>
+          <t>167.735 to 189.064</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>857.601 to 940.653</t>
+          <t>848.203 to 891.262</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3959.83 to 15961.5</t>
+          <t>3067.06 to 6818.42</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.0127772 to 0.051503</t>
+          <t>0.0299106 to 0.0664946</t>
         </is>
       </c>
     </row>
@@ -1311,16 +1311,16 @@
         <v>36</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>184.057 to 207.364</t>
+          <t>166.228 to 182.943</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>873.715 to 966.46</t>
+          <t>836.212 to 881.517</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">

</xml_diff>